<commit_message>
se agrega cartera en el formato modular
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IRISCENE ENGINEERING CORPORATION SLU\Data Analytics Reporting Fractalia - CHILE\Miguel Paredes\Desarrollo\02. PYTHON\202_bot_jira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3634CEE3-48C8-41FB-9CF6-86553A2ABE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F029AF-BCB0-45AD-902B-C73E1F5321BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="92">
   <si>
     <t>Ticket</t>
   </si>
@@ -65,159 +65,159 @@
     <t>Descarga insumos SF</t>
   </si>
   <si>
+    <t>Sí (02/09/2026 09:00)</t>
+  </si>
+  <si>
+    <t>510252</t>
+  </si>
+  <si>
     <t>DSS-9337</t>
   </si>
   <si>
+    <t>Reestructuración crudos</t>
+  </si>
+  <si>
+    <t>510339</t>
+  </si>
+  <si>
     <t>Daily</t>
   </si>
   <si>
+    <t>510253</t>
+  </si>
+  <si>
+    <t>510254</t>
+  </si>
+  <si>
+    <t>Reunion equipo: Revisión Audit dependencias BPO CHILE</t>
+  </si>
+  <si>
+    <t>510340</t>
+  </si>
+  <si>
+    <t>Corrida ETL tráfico, calidad, usuarios chile</t>
+  </si>
+  <si>
+    <t>510341</t>
+  </si>
+  <si>
+    <t>510342</t>
+  </si>
+  <si>
+    <t>510255</t>
+  </si>
+  <si>
+    <t>510256</t>
+  </si>
+  <si>
     <t>Seguimiento Reestructuración Ecosistema Reporting</t>
   </si>
   <si>
+    <t>510343</t>
+  </si>
+  <si>
+    <t>Sí (04/09/2026 10:11)</t>
+  </si>
+  <si>
+    <t>511015</t>
+  </si>
+  <si>
+    <t>Actualizacion CDM agosto</t>
+  </si>
+  <si>
+    <t>510979</t>
+  </si>
+  <si>
+    <t>510980</t>
+  </si>
+  <si>
+    <t>510981</t>
+  </si>
+  <si>
+    <t>511016</t>
+  </si>
+  <si>
+    <t>Reunión cliente: Accesos y servidor chile</t>
+  </si>
+  <si>
+    <t>510982</t>
+  </si>
+  <si>
+    <t>511017</t>
+  </si>
+  <si>
+    <t>511018</t>
+  </si>
+  <si>
+    <t>510983</t>
+  </si>
+  <si>
+    <t>511019</t>
+  </si>
+  <si>
+    <t>510984</t>
+  </si>
+  <si>
+    <t>511020</t>
+  </si>
+  <si>
+    <t>511021</t>
+  </si>
+  <si>
+    <t>Actualizacion Cuartiles agosto</t>
+  </si>
+  <si>
+    <t>510985</t>
+  </si>
+  <si>
+    <t>511022</t>
+  </si>
+  <si>
+    <t>Reunion: Afinación Ruta de trabajo BPO CHILE</t>
+  </si>
+  <si>
+    <t>510986</t>
+  </si>
+  <si>
+    <t>511023</t>
+  </si>
+  <si>
+    <t>510987</t>
+  </si>
+  <si>
+    <t>DSS-9712</t>
+  </si>
+  <si>
+    <t>Extraccion de datos, query</t>
+  </si>
+  <si>
+    <t>510988</t>
+  </si>
+  <si>
+    <t>511024</t>
+  </si>
+  <si>
+    <t>511025</t>
+  </si>
+  <si>
+    <t>Se termina de modelar el archivo para el envío</t>
+  </si>
+  <si>
+    <t>511026</t>
+  </si>
+  <si>
+    <t>511027</t>
+  </si>
+  <si>
+    <t>Registro de tickets</t>
+  </si>
+  <si>
+    <t>510989</t>
+  </si>
+  <si>
     <t>Envío ISN</t>
   </si>
   <si>
-    <t>Registro de tickets</t>
-  </si>
-  <si>
-    <t>Sí (02/09/2026 09:00)</t>
-  </si>
-  <si>
-    <t>510252</t>
-  </si>
-  <si>
-    <t>Reestructuración crudos</t>
-  </si>
-  <si>
-    <t>510339</t>
-  </si>
-  <si>
-    <t>510253</t>
-  </si>
-  <si>
-    <t>510254</t>
-  </si>
-  <si>
-    <t>Reunion equipo: Revisión Audit dependencias BPO CHILE</t>
-  </si>
-  <si>
-    <t>510340</t>
-  </si>
-  <si>
-    <t>Corrida ETL tráfico, calidad, usuarios chile</t>
-  </si>
-  <si>
-    <t>510341</t>
-  </si>
-  <si>
-    <t>510342</t>
-  </si>
-  <si>
-    <t>510255</t>
-  </si>
-  <si>
-    <t>510256</t>
-  </si>
-  <si>
-    <t>510343</t>
-  </si>
-  <si>
-    <t>Sí (04/09/2026 10:11)</t>
-  </si>
-  <si>
-    <t>511015</t>
-  </si>
-  <si>
-    <t>Actualizacion CDM agosto</t>
-  </si>
-  <si>
-    <t>510979</t>
-  </si>
-  <si>
-    <t>510980</t>
-  </si>
-  <si>
-    <t>510981</t>
-  </si>
-  <si>
-    <t>511016</t>
-  </si>
-  <si>
-    <t>Reunión cliente: Accesos y servidor chile</t>
-  </si>
-  <si>
-    <t>510982</t>
-  </si>
-  <si>
-    <t>511017</t>
-  </si>
-  <si>
-    <t>511018</t>
-  </si>
-  <si>
-    <t>510983</t>
-  </si>
-  <si>
-    <t>511019</t>
-  </si>
-  <si>
-    <t>510984</t>
-  </si>
-  <si>
-    <t>511020</t>
-  </si>
-  <si>
-    <t>511021</t>
-  </si>
-  <si>
-    <t>Actualizacion Cuartiles agosto</t>
-  </si>
-  <si>
-    <t>510985</t>
-  </si>
-  <si>
-    <t>511022</t>
-  </si>
-  <si>
-    <t>Reunion: Afinación Ruta de trabajo BPO CHILE</t>
-  </si>
-  <si>
-    <t>510986</t>
-  </si>
-  <si>
-    <t>511023</t>
-  </si>
-  <si>
-    <t>510987</t>
-  </si>
-  <si>
-    <t>DSS-9712</t>
-  </si>
-  <si>
-    <t>Extraccion de datos, query</t>
-  </si>
-  <si>
-    <t>510988</t>
-  </si>
-  <si>
-    <t>511024</t>
-  </si>
-  <si>
-    <t>511025</t>
-  </si>
-  <si>
-    <t>Se termina de modelar el archivo para el envío</t>
-  </si>
-  <si>
-    <t>511026</t>
-  </si>
-  <si>
-    <t>511027</t>
-  </si>
-  <si>
-    <t>510989</t>
-  </si>
-  <si>
     <t>Sí (07/09/2026 08:15)</t>
   </si>
   <si>
@@ -254,7 +254,61 @@
     <t>511400</t>
   </si>
   <si>
+    <t>Sí (08/09/2026 09:05)</t>
+  </si>
+  <si>
+    <t>511692</t>
+  </si>
+  <si>
+    <t>Migración cartera a python</t>
+  </si>
+  <si>
+    <t>511812</t>
+  </si>
+  <si>
+    <t>511813</t>
+  </si>
+  <si>
+    <t>511814</t>
+  </si>
+  <si>
     <t>Solicitud de archivos actualizados de comentaros y descripciones salesforce</t>
+  </si>
+  <si>
+    <t>511815</t>
+  </si>
+  <si>
+    <t>511693</t>
+  </si>
+  <si>
+    <t>511694</t>
+  </si>
+  <si>
+    <t>DSS-9721</t>
+  </si>
+  <si>
+    <t>Elaboracion factura julio</t>
+  </si>
+  <si>
+    <t>511816</t>
+  </si>
+  <si>
+    <t>511695</t>
+  </si>
+  <si>
+    <t>511696</t>
+  </si>
+  <si>
+    <t>DSS-9722</t>
+  </si>
+  <si>
+    <t>Elaboracion factura agosto</t>
+  </si>
+  <si>
+    <t>revision onedrive</t>
+  </si>
+  <si>
+    <t>Inventario de Informes BPO Chile</t>
   </si>
 </sst>
 </file>
@@ -343,16 +397,16 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <top style="thin">
+        <bottom style="thin">
           <color auto="1"/>
-        </top>
+        </bottom>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
+        <top style="thin">
           <color auto="1"/>
-        </bottom>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -394,8 +448,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H44" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:H44" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H60" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="3" tableBorderDxfId="4">
+  <autoFilter ref="A1:H60" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ticket"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="2"/>
@@ -697,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
@@ -753,15 +807,15 @@
         <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1">
         <v>46266.336805555547</v>
@@ -774,18 +828,18 @@
         <v>46266.374999999993</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1">
         <v>46266.375</v>
@@ -798,18 +852,18 @@
         <v>46266.388888888891</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1">
         <v>46266.388888888891</v>
@@ -822,18 +876,18 @@
         <v>46266.395833333336</v>
       </c>
       <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
         <v>17</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1">
         <v>46266.395833333343</v>
@@ -846,13 +900,13 @@
         <v>46266.465277777788</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -870,18 +924,18 @@
         <v>46266.479166666672</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B8" s="1">
         <v>46266.479166666657</v>
@@ -894,13 +948,13 @@
         <v>46266.583333333321</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -921,15 +975,15 @@
         <v>9</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B10" s="1">
         <v>46266.628472222219</v>
@@ -942,18 +996,18 @@
         <v>46266.708333333328</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1">
         <v>46266.708333333343</v>
@@ -966,13 +1020,13 @@
         <v>46266.770833333343</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -993,10 +1047,10 @@
         <v>9</v>
       </c>
       <c r="G12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1014,18 +1068,18 @@
         <v>46267.374999999993</v>
       </c>
       <c r="E13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1">
         <v>46267.375</v>
@@ -1038,13 +1092,13 @@
         <v>46267.392361111109</v>
       </c>
       <c r="E14" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1062,13 +1116,13 @@
         <v>46267.465277777774</v>
       </c>
       <c r="E15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1086,13 +1140,13 @@
         <v>46267.479166666672</v>
       </c>
       <c r="E16" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G16" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1110,13 +1164,13 @@
         <v>46267.524305555547</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G17" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -1134,13 +1188,13 @@
         <v>46267.583333333328</v>
       </c>
       <c r="E18" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1161,10 +1215,10 @@
         <v>9</v>
       </c>
       <c r="G19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H19" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1182,18 +1236,18 @@
         <v>46267.708333333328</v>
       </c>
       <c r="E20" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B21" s="1">
         <v>46267.708333333343</v>
@@ -1206,13 +1260,13 @@
         <v>46267.770833333343</v>
       </c>
       <c r="E21" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G21" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,10 +1287,10 @@
         <v>9</v>
       </c>
       <c r="G22" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H22" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -1254,18 +1308,18 @@
         <v>46268.374999999993</v>
       </c>
       <c r="E23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H23" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B24" s="1">
         <v>46268.375</v>
@@ -1278,13 +1332,13 @@
         <v>46268.385416666664</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H24" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1302,13 +1356,13 @@
         <v>46268.465277777766</v>
       </c>
       <c r="E25" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G25" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H25" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1326,18 +1380,18 @@
         <v>46268.479166666672</v>
       </c>
       <c r="E26" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G26" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H26" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B27" s="1">
         <v>46268.479166666657</v>
@@ -1350,13 +1404,13 @@
         <v>46268.548611111102</v>
       </c>
       <c r="E27" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G27" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H27" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -1374,13 +1428,13 @@
         <v>46268.583333333328</v>
       </c>
       <c r="E28" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G28" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -1401,15 +1455,15 @@
         <v>9</v>
       </c>
       <c r="G29" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B30" s="1">
         <v>46268.628472222219</v>
@@ -1422,18 +1476,18 @@
         <v>46268.708333333328</v>
       </c>
       <c r="E30" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G30" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H30" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B31" s="1">
         <v>46268.708333333343</v>
@@ -1446,13 +1500,13 @@
         <v>46268.770833333343</v>
       </c>
       <c r="E31" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G31" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1473,15 +1527,15 @@
         <v>9</v>
       </c>
       <c r="G32" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H32" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B33" s="1">
         <v>46269.336805555547</v>
@@ -1494,18 +1548,18 @@
         <v>46269.374999999993</v>
       </c>
       <c r="E33" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G33" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B34" s="1">
         <v>46269.375</v>
@@ -1518,18 +1572,18 @@
         <v>46269.392361111109</v>
       </c>
       <c r="E34" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G34" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H34" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B35" s="1">
         <v>46269.392361111109</v>
@@ -1542,13 +1596,13 @@
         <v>46269.422916666663</v>
       </c>
       <c r="E35" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="G35" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -1566,7 +1620,7 @@
         <v>46269.440972222226</v>
       </c>
       <c r="E36" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="G36" t="s">
         <v>61</v>
@@ -1614,7 +1668,7 @@
         <v>46269.472222222234</v>
       </c>
       <c r="E38" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G38" t="s">
         <v>61</v>
@@ -1673,7 +1727,7 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B41" s="1">
         <v>46269.628472222219</v>
@@ -1686,7 +1740,7 @@
         <v>46269.666666666664</v>
       </c>
       <c r="E41" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G41" t="s">
         <v>61</v>
@@ -1697,7 +1751,7 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B42" s="1">
         <v>46269.666666666657</v>
@@ -1710,7 +1764,7 @@
         <v>46269.708333333321</v>
       </c>
       <c r="E42" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="G42" t="s">
         <v>61</v>
@@ -1721,7 +1775,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B43" s="1">
         <v>46269.708333333343</v>
@@ -1748,17 +1802,365 @@
         <v>8</v>
       </c>
       <c r="B44" s="1">
-        <v>46272.430555555555</v>
+        <v>46272.333333333343</v>
       </c>
       <c r="C44" s="3">
-        <v>6.9444444444444441E-3</v>
+        <v>3.472222222222222E-3</v>
       </c>
       <c r="D44" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.336805555562</v>
+      </c>
+      <c r="E44" t="s">
+        <v>9</v>
+      </c>
+      <c r="G44" t="s">
+        <v>73</v>
+      </c>
+      <c r="H44" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="1">
+        <v>46272.336805555547</v>
+      </c>
+      <c r="C45" s="3">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="D45" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.374999999993</v>
+      </c>
+      <c r="E45" t="s">
+        <v>75</v>
+      </c>
+      <c r="G45" t="s">
+        <v>73</v>
+      </c>
+      <c r="H45" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="1">
+        <v>46272.375</v>
+      </c>
+      <c r="C46" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D46" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.385416666664</v>
+      </c>
+      <c r="E46" t="s">
+        <v>15</v>
+      </c>
+      <c r="G46" t="s">
+        <v>73</v>
+      </c>
+      <c r="H46" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47" s="1">
+        <v>46272.385416666657</v>
+      </c>
+      <c r="C47" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D47" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.427083333321</v>
+      </c>
+      <c r="E47" t="s">
+        <v>75</v>
+      </c>
+      <c r="G47" t="s">
+        <v>73</v>
+      </c>
+      <c r="H47" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>8</v>
+      </c>
+      <c r="B48" s="1">
+        <v>46272.427083333343</v>
+      </c>
+      <c r="C48" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D48" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.437500000007</v>
+      </c>
+      <c r="E48" t="s">
+        <v>79</v>
+      </c>
+      <c r="G48" t="s">
+        <v>73</v>
+      </c>
+      <c r="H48" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>12</v>
+      </c>
+      <c r="B49" s="1">
         <v>46272.4375</v>
       </c>
-      <c r="E44" t="s">
+      <c r="C49" s="3">
+        <v>0.14583333333333329</v>
+      </c>
+      <c r="D49" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.583333333336</v>
+      </c>
+      <c r="E49" t="s">
+        <v>75</v>
+      </c>
+      <c r="G49" t="s">
         <v>73</v>
+      </c>
+      <c r="H49" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>8</v>
+      </c>
+      <c r="B50" s="1">
+        <v>46272.625</v>
+      </c>
+      <c r="C50" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D50" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.628472222219</v>
+      </c>
+      <c r="E50" t="s">
+        <v>9</v>
+      </c>
+      <c r="G50" t="s">
+        <v>73</v>
+      </c>
+      <c r="H50" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>83</v>
+      </c>
+      <c r="B51" s="1">
+        <v>46272.628472222219</v>
+      </c>
+      <c r="C51" s="3">
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="D51" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.708333333328</v>
+      </c>
+      <c r="E51" t="s">
+        <v>84</v>
+      </c>
+      <c r="G51" t="s">
+        <v>73</v>
+      </c>
+      <c r="H51" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>12</v>
+      </c>
+      <c r="B52" s="1">
+        <v>46272.708333333343</v>
+      </c>
+      <c r="C52" s="3">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D52" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.763888888898</v>
+      </c>
+      <c r="E52" t="s">
+        <v>25</v>
+      </c>
+      <c r="G52" t="s">
+        <v>73</v>
+      </c>
+      <c r="H52" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>83</v>
+      </c>
+      <c r="B53" s="1">
+        <v>46272.763888888891</v>
+      </c>
+      <c r="C53" s="3">
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="D53" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46272.776388888888</v>
+      </c>
+      <c r="E53" t="s">
+        <v>84</v>
+      </c>
+      <c r="G53" t="s">
+        <v>73</v>
+      </c>
+      <c r="H53" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54" s="1">
+        <v>46273.333333333336</v>
+      </c>
+      <c r="C54" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D54" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.336805555555</v>
+      </c>
+      <c r="E54" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>12</v>
+      </c>
+      <c r="B55" s="1">
+        <v>46273.375</v>
+      </c>
+      <c r="C55" s="3">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D55" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.388888888891</v>
+      </c>
+      <c r="E55" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>88</v>
+      </c>
+      <c r="B56" s="1">
+        <v>46273.388888888891</v>
+      </c>
+      <c r="C56" s="3">
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="D56" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.401388888888</v>
+      </c>
+      <c r="E56" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57" s="1">
+        <v>46273.395833333336</v>
+      </c>
+      <c r="C57" s="3">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="D57" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.40625</v>
+      </c>
+      <c r="E57" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>12</v>
+      </c>
+      <c r="B58" s="1">
+        <v>46273.479166666664</v>
+      </c>
+      <c r="C58" s="3">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D58" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.5</v>
+      </c>
+      <c r="E58" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>8</v>
+      </c>
+      <c r="B59" s="1">
+        <v>46273.520833333336</v>
+      </c>
+      <c r="C59" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D59" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.583333333336</v>
+      </c>
+      <c r="E59" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>12</v>
+      </c>
+      <c r="B60" s="1">
+        <v>46273.708333333336</v>
+      </c>
+      <c r="C60" s="3">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D60" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.763888888891</v>
+      </c>
+      <c r="E60" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agregado usuarios, notas de credito
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IRISCENE ENGINEERING CORPORATION SLU\Data Analytics Reporting Fractalia - CHILE\Miguel Paredes\Desarrollo\02. PYTHON\202_bot_jira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F029AF-BCB0-45AD-902B-C73E1F5321BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301DD301-6329-48CA-817D-1F79D44B05AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="158">
   <si>
     <t>Ticket</t>
   </si>
@@ -299,16 +300,214 @@
     <t>511696</t>
   </si>
   <si>
+    <t>Sí (10/09/2026 09:05)</t>
+  </si>
+  <si>
+    <t>512653</t>
+  </si>
+  <si>
     <t>DSS-9722</t>
   </si>
   <si>
     <t>Elaboracion factura agosto</t>
   </si>
   <si>
+    <t>512382</t>
+  </si>
+  <si>
+    <t>512383</t>
+  </si>
+  <si>
+    <t>512384</t>
+  </si>
+  <si>
     <t>revision onedrive</t>
   </si>
   <si>
+    <t>512385</t>
+  </si>
+  <si>
+    <t>512654</t>
+  </si>
+  <si>
+    <t>512386</t>
+  </si>
+  <si>
+    <t>512655</t>
+  </si>
+  <si>
     <t>Inventario de Informes BPO Chile</t>
+  </si>
+  <si>
+    <t>Sí (10/09/2026 09:06)</t>
+  </si>
+  <si>
+    <t>512656</t>
+  </si>
+  <si>
+    <t>512387</t>
+  </si>
+  <si>
+    <t>A pedido de Karen se agrego en el landing el tablero de control telefonica chile</t>
+  </si>
+  <si>
+    <t>512657</t>
+  </si>
+  <si>
+    <t>A pedido de Karen se agrego en el landing el informe de gestion back y front</t>
+  </si>
+  <si>
+    <t>512658</t>
+  </si>
+  <si>
+    <t>512659</t>
+  </si>
+  <si>
+    <t>512388</t>
+  </si>
+  <si>
+    <t>512660</t>
+  </si>
+  <si>
+    <t>Reunion: revisión factura agosto</t>
+  </si>
+  <si>
+    <t>512661</t>
+  </si>
+  <si>
+    <t>512389</t>
+  </si>
+  <si>
+    <t>512662</t>
+  </si>
+  <si>
+    <t>512390</t>
+  </si>
+  <si>
+    <t>512391</t>
+  </si>
+  <si>
+    <t>a solicitud de oscar se tabaja en: "Inventario de Informes Repositorio BI"</t>
+  </si>
+  <si>
+    <t>512663</t>
+  </si>
+  <si>
+    <t>512664</t>
+  </si>
+  <si>
+    <t>Migracion cartera</t>
+  </si>
+  <si>
+    <t>512392</t>
+  </si>
+  <si>
+    <t>512393</t>
+  </si>
+  <si>
+    <t>Revision migracion procesos crudos</t>
+  </si>
+  <si>
+    <t>512394</t>
+  </si>
+  <si>
+    <t>Sí (11/09/2026 08:37)</t>
+  </si>
+  <si>
+    <t>512980</t>
+  </si>
+  <si>
+    <t>Análisis factura agosto</t>
+  </si>
+  <si>
+    <t>512981</t>
+  </si>
+  <si>
+    <t>513014</t>
+  </si>
+  <si>
+    <t>Revision de factura julio por confirmación del cliente</t>
+  </si>
+  <si>
+    <t>512982</t>
+  </si>
+  <si>
+    <t>512983</t>
+  </si>
+  <si>
+    <t>513015</t>
+  </si>
+  <si>
+    <t>Llamada andrea sobre la factura de agosto</t>
+  </si>
+  <si>
+    <t>512984</t>
+  </si>
+  <si>
+    <t>Revision de horarios de actualización para procesos de informes migrados</t>
+  </si>
+  <si>
+    <t>513016</t>
+  </si>
+  <si>
+    <t>512985</t>
+  </si>
+  <si>
+    <t>Corrida ETL tráfico, calidad, usuarios chile (Reproceso por muestreo de IA calidad)</t>
+  </si>
+  <si>
+    <t>512986</t>
+  </si>
+  <si>
+    <t>513017</t>
+  </si>
+  <si>
+    <t>Reunion con carlos: Revisión BPO Chile To address</t>
+  </si>
+  <si>
+    <t>513018</t>
+  </si>
+  <si>
+    <t>512987</t>
+  </si>
+  <si>
+    <t>512988</t>
+  </si>
+  <si>
+    <t>513019</t>
+  </si>
+  <si>
+    <t>Ingreso de horas día anterior</t>
+  </si>
+  <si>
+    <t>513020</t>
+  </si>
+  <si>
+    <t>Envío de maqueta al cliente</t>
+  </si>
+  <si>
+    <t>Envío cambios SM</t>
+  </si>
+  <si>
+    <t>Envío dimensionado</t>
+  </si>
+  <si>
+    <t>Modificacion de documentos programacion por tablas</t>
+  </si>
+  <si>
+    <t>DSS-9734</t>
+  </si>
+  <si>
+    <t>DSS-9737</t>
+  </si>
+  <si>
+    <t>Se revisó lo solicitado y se validó que la respuesta de bi es correcta.</t>
+  </si>
+  <si>
+    <t>Se revisó lo solicitado y se validó que la respuesta de bi es correcta error en la operación por la bd_general.</t>
+  </si>
+  <si>
+    <t>DSS-9735</t>
   </si>
 </sst>
 </file>
@@ -448,8 +647,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H60" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="3" tableBorderDxfId="4">
-  <autoFilter ref="A1:H60" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H105" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="3" tableBorderDxfId="4">
+  <autoFilter ref="A1:H105" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ticket"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="2"/>
@@ -751,7 +950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
@@ -2042,71 +2241,95 @@
         <v>8</v>
       </c>
       <c r="B54" s="1">
-        <v>46273.333333333336</v>
+        <v>46273.333333333343</v>
       </c>
       <c r="C54" s="3">
         <v>3.472222222222222E-3</v>
       </c>
       <c r="D54" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.336805555555</v>
+        <v>46273.336805555562</v>
       </c>
       <c r="E54" t="s">
         <v>9</v>
       </c>
+      <c r="G54" t="s">
+        <v>88</v>
+      </c>
+      <c r="H54" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="B55" s="1">
-        <v>46273.375</v>
+        <v>46273.336805555547</v>
       </c>
       <c r="C55" s="3">
-        <v>1.3888888888888888E-2</v>
+        <v>3.8194444444444448E-2</v>
       </c>
       <c r="D55" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.388888888891</v>
+        <v>46273.374999999993</v>
       </c>
       <c r="E55" t="s">
-        <v>15</v>
+        <v>91</v>
+      </c>
+      <c r="G55" t="s">
+        <v>88</v>
+      </c>
+      <c r="H55" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>12</v>
+      </c>
+      <c r="B56" s="1">
+        <v>46273.375</v>
+      </c>
+      <c r="C56" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D56" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.388888888891</v>
+      </c>
+      <c r="E56" t="s">
+        <v>15</v>
+      </c>
+      <c r="G56" t="s">
         <v>88</v>
       </c>
-      <c r="B56" s="1">
-        <v>46273.388888888891</v>
-      </c>
-      <c r="C56" s="3">
-        <v>1.2500000000000001E-2</v>
-      </c>
-      <c r="D56" s="3">
-        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.401388888888</v>
-      </c>
-      <c r="E56" t="s">
-        <v>89</v>
+      <c r="H56" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="B57" s="1">
+        <v>46273.388888888891</v>
+      </c>
+      <c r="C57" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D57" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
         <v>46273.395833333336</v>
       </c>
-      <c r="C57" s="3">
-        <v>1.0416666666666666E-2</v>
-      </c>
-      <c r="D57" s="3">
-        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.40625</v>
-      </c>
       <c r="E57" t="s">
-        <v>90</v>
+        <v>91</v>
+      </c>
+      <c r="G57" t="s">
+        <v>88</v>
+      </c>
+      <c r="H57" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -2114,53 +2337,1080 @@
         <v>12</v>
       </c>
       <c r="B58" s="1">
-        <v>46273.479166666664</v>
+        <v>46273.395833333343</v>
       </c>
       <c r="C58" s="3">
-        <v>2.0833333333333332E-2</v>
+        <v>1.041666666666667E-2</v>
       </c>
       <c r="D58" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.5</v>
+        <v>46273.406250000007</v>
       </c>
       <c r="E58" t="s">
-        <v>90</v>
+        <v>95</v>
+      </c>
+      <c r="G58" t="s">
+        <v>88</v>
+      </c>
+      <c r="H58" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="B59" s="1">
-        <v>46273.520833333336</v>
+        <v>46273.40625</v>
       </c>
       <c r="C59" s="3">
-        <v>6.25E-2</v>
+        <v>7.2916666666666671E-2</v>
       </c>
       <c r="D59" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.583333333336</v>
+        <v>46273.479166666664</v>
       </c>
       <c r="E59" t="s">
         <v>91</v>
       </c>
+      <c r="G59" t="s">
+        <v>88</v>
+      </c>
+      <c r="H59" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>12</v>
       </c>
       <c r="B60" s="1">
-        <v>46273.708333333336</v>
+        <v>46273.479166666657</v>
       </c>
       <c r="C60" s="3">
-        <v>5.5555555555555552E-2</v>
+        <v>2.0833333333333329E-2</v>
       </c>
       <c r="D60" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46273.763888888891</v>
+        <v>46273.499999999993</v>
       </c>
       <c r="E60" t="s">
+        <v>95</v>
+      </c>
+      <c r="G60" t="s">
+        <v>88</v>
+      </c>
+      <c r="H60" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>90</v>
+      </c>
+      <c r="B61" s="1">
+        <v>46273.5</v>
+      </c>
+      <c r="C61" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D61" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.520833333336</v>
+      </c>
+      <c r="E61" t="s">
+        <v>91</v>
+      </c>
+      <c r="G61" t="s">
+        <v>88</v>
+      </c>
+      <c r="H61" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>8</v>
+      </c>
+      <c r="B62" s="1">
+        <v>46273.520833333343</v>
+      </c>
+      <c r="C62" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D62" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.583333333343</v>
+      </c>
+      <c r="E62" t="s">
+        <v>100</v>
+      </c>
+      <c r="G62" t="s">
+        <v>101</v>
+      </c>
+      <c r="H62" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>8</v>
+      </c>
+      <c r="B63" s="1">
+        <v>46273.625</v>
+      </c>
+      <c r="C63" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D63" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.628472222219</v>
+      </c>
+      <c r="E63" t="s">
+        <v>9</v>
+      </c>
+      <c r="G63" t="s">
+        <v>101</v>
+      </c>
+      <c r="H63" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>8</v>
+      </c>
+      <c r="B64" s="1">
+        <v>46273.628472222219</v>
+      </c>
+      <c r="C64" s="3">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="D64" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.666666666664</v>
+      </c>
+      <c r="E64" t="s">
+        <v>104</v>
+      </c>
+      <c r="G64" t="s">
+        <v>101</v>
+      </c>
+      <c r="H64" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>8</v>
+      </c>
+      <c r="B65" s="1">
+        <v>46273.666666666657</v>
+      </c>
+      <c r="C65" s="3">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="D65" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.708333333321</v>
+      </c>
+      <c r="E65" t="s">
+        <v>106</v>
+      </c>
+      <c r="G65" t="s">
+        <v>101</v>
+      </c>
+      <c r="H65" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>12</v>
+      </c>
+      <c r="B66" s="1">
+        <v>46273.708333333343</v>
+      </c>
+      <c r="C66" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D66" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46273.770833333343</v>
+      </c>
+      <c r="E66" t="s">
         <v>25</v>
+      </c>
+      <c r="G66" t="s">
+        <v>101</v>
+      </c>
+      <c r="H66" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>8</v>
+      </c>
+      <c r="B67" s="1">
+        <v>46274.333333333343</v>
+      </c>
+      <c r="C67" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D67" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.336805555562</v>
+      </c>
+      <c r="E67" t="s">
+        <v>9</v>
+      </c>
+      <c r="G67" t="s">
+        <v>101</v>
+      </c>
+      <c r="H67" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>90</v>
+      </c>
+      <c r="B68" s="1">
+        <v>46274.336805555547</v>
+      </c>
+      <c r="C68" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D68" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.347222222212</v>
+      </c>
+      <c r="E68" t="s">
+        <v>91</v>
+      </c>
+      <c r="G68" t="s">
+        <v>101</v>
+      </c>
+      <c r="H68" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>90</v>
+      </c>
+      <c r="B69" s="1">
+        <v>46274.347222222219</v>
+      </c>
+      <c r="C69" s="3">
+        <v>2.4305555555555559E-2</v>
+      </c>
+      <c r="D69" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.371527777774</v>
+      </c>
+      <c r="E69" t="s">
+        <v>111</v>
+      </c>
+      <c r="G69" t="s">
+        <v>101</v>
+      </c>
+      <c r="H69" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>90</v>
+      </c>
+      <c r="B70" s="1">
+        <v>46274.371527777781</v>
+      </c>
+      <c r="C70" s="3">
+        <v>3.4722222222222217E-2</v>
+      </c>
+      <c r="D70" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.40625</v>
+      </c>
+      <c r="E70" t="s">
+        <v>91</v>
+      </c>
+      <c r="G70" t="s">
+        <v>101</v>
+      </c>
+      <c r="H70" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>90</v>
+      </c>
+      <c r="B71" s="1">
+        <v>46274.40625</v>
+      </c>
+      <c r="C71" s="3">
+        <v>1.041666666666667E-2</v>
+      </c>
+      <c r="D71" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.416666666664</v>
+      </c>
+      <c r="E71" t="s">
+        <v>111</v>
+      </c>
+      <c r="G71" t="s">
+        <v>101</v>
+      </c>
+      <c r="H71" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>12</v>
+      </c>
+      <c r="B72" s="1">
+        <v>46274.416666666657</v>
+      </c>
+      <c r="C72" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D72" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.430555555547</v>
+      </c>
+      <c r="E72" t="s">
+        <v>15</v>
+      </c>
+      <c r="G72" t="s">
+        <v>101</v>
+      </c>
+      <c r="H72" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>90</v>
+      </c>
+      <c r="B73" s="1">
+        <v>46274.430555555547</v>
+      </c>
+      <c r="C73" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D73" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.444444444438</v>
+      </c>
+      <c r="E73" t="s">
+        <v>91</v>
+      </c>
+      <c r="G73" t="s">
+        <v>101</v>
+      </c>
+      <c r="H73" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>12</v>
+      </c>
+      <c r="B74" s="1">
+        <v>46274.444444444453</v>
+      </c>
+      <c r="C74" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D74" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.458333333343</v>
+      </c>
+      <c r="E74" t="s">
+        <v>117</v>
+      </c>
+      <c r="G74" t="s">
+        <v>101</v>
+      </c>
+      <c r="H74" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>8</v>
+      </c>
+      <c r="B75" s="1">
+        <v>46274.458333333343</v>
+      </c>
+      <c r="C75" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D75" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.472222222234</v>
+      </c>
+      <c r="E75" t="s">
+        <v>20</v>
+      </c>
+      <c r="G75" t="s">
+        <v>101</v>
+      </c>
+      <c r="H75" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" s="1">
+        <v>46274.472222222219</v>
+      </c>
+      <c r="C76" s="3">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="D76" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.583333333328</v>
+      </c>
+      <c r="E76" t="s">
+        <v>120</v>
+      </c>
+      <c r="G76" t="s">
+        <v>101</v>
+      </c>
+      <c r="H76" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>8</v>
+      </c>
+      <c r="B77" s="1">
+        <v>46274.625</v>
+      </c>
+      <c r="C77" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D77" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.628472222219</v>
+      </c>
+      <c r="E77" t="s">
+        <v>9</v>
+      </c>
+      <c r="G77" t="s">
+        <v>101</v>
+      </c>
+      <c r="H77" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>12</v>
+      </c>
+      <c r="B78" s="1">
+        <v>46274.628472222219</v>
+      </c>
+      <c r="C78" s="3">
+        <v>0.1423611111111111</v>
+      </c>
+      <c r="D78" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46274.770833333328</v>
+      </c>
+      <c r="E78" t="s">
+        <v>123</v>
+      </c>
+      <c r="G78" t="s">
+        <v>101</v>
+      </c>
+      <c r="H78" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>8</v>
+      </c>
+      <c r="B79" s="1">
+        <v>46275.333333333343</v>
+      </c>
+      <c r="C79" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D79" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.336805555562</v>
+      </c>
+      <c r="E79" t="s">
+        <v>9</v>
+      </c>
+      <c r="G79" t="s">
+        <v>125</v>
+      </c>
+      <c r="H79" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>90</v>
+      </c>
+      <c r="B80" s="1">
+        <v>46275.336805555547</v>
+      </c>
+      <c r="C80" s="3">
+        <v>3.8194444444444448E-2</v>
+      </c>
+      <c r="D80" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.374999999993</v>
+      </c>
+      <c r="E80" t="s">
+        <v>127</v>
+      </c>
+      <c r="G80" t="s">
+        <v>125</v>
+      </c>
+      <c r="H80" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>12</v>
+      </c>
+      <c r="B81" s="1">
+        <v>46275.375</v>
+      </c>
+      <c r="C81" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D81" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.395833333336</v>
+      </c>
+      <c r="E81" t="s">
+        <v>15</v>
+      </c>
+      <c r="G81" t="s">
+        <v>125</v>
+      </c>
+      <c r="H81" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>83</v>
+      </c>
+      <c r="B82" s="1">
+        <v>46275.395833333343</v>
+      </c>
+      <c r="C82" s="3">
+        <v>7.9861111111111105E-2</v>
+      </c>
+      <c r="D82" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.475694444453</v>
+      </c>
+      <c r="E82" t="s">
+        <v>130</v>
+      </c>
+      <c r="G82" t="s">
+        <v>125</v>
+      </c>
+      <c r="H82" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>8</v>
+      </c>
+      <c r="B83" s="1">
+        <v>46275.475694444453</v>
+      </c>
+      <c r="C83" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D83" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.489583333343</v>
+      </c>
+      <c r="E83" t="s">
+        <v>20</v>
+      </c>
+      <c r="G83" t="s">
+        <v>125</v>
+      </c>
+      <c r="H83" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>90</v>
+      </c>
+      <c r="B84" s="1">
+        <v>46275.489583333343</v>
+      </c>
+      <c r="C84" s="3">
+        <v>3.4722222222222217E-2</v>
+      </c>
+      <c r="D84" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.524305555562</v>
+      </c>
+      <c r="E84" t="s">
+        <v>127</v>
+      </c>
+      <c r="G84" t="s">
+        <v>125</v>
+      </c>
+      <c r="H84" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>8</v>
+      </c>
+      <c r="B85" s="1">
+        <v>46275.524305555547</v>
+      </c>
+      <c r="C85" s="3">
+        <v>4.1666666666666666E-3</v>
+      </c>
+      <c r="D85" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.528472222213</v>
+      </c>
+      <c r="E85" t="s">
+        <v>134</v>
+      </c>
+      <c r="G85" t="s">
+        <v>125</v>
+      </c>
+      <c r="H85" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>12</v>
+      </c>
+      <c r="B86" s="1">
+        <v>46275.52847222222</v>
+      </c>
+      <c r="C86" s="3">
+        <v>5.486111111111111E-2</v>
+      </c>
+      <c r="D86" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.583333333328</v>
+      </c>
+      <c r="E86" t="s">
+        <v>136</v>
+      </c>
+      <c r="G86" t="s">
+        <v>125</v>
+      </c>
+      <c r="H86" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>8</v>
+      </c>
+      <c r="B87" s="1">
+        <v>46275.625</v>
+      </c>
+      <c r="C87" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D87" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.628472222219</v>
+      </c>
+      <c r="E87" t="s">
+        <v>9</v>
+      </c>
+      <c r="G87" t="s">
+        <v>125</v>
+      </c>
+      <c r="H87" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>8</v>
+      </c>
+      <c r="B88" s="1">
+        <v>46275.628472222219</v>
+      </c>
+      <c r="C88" s="3">
+        <v>1.388888888888889E-2</v>
+      </c>
+      <c r="D88" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.642361111109</v>
+      </c>
+      <c r="E88" t="s">
+        <v>139</v>
+      </c>
+      <c r="G88" t="s">
+        <v>125</v>
+      </c>
+      <c r="H88" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>90</v>
+      </c>
+      <c r="B89" s="1">
+        <v>46275.642361111109</v>
+      </c>
+      <c r="C89" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D89" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.649305555555</v>
+      </c>
+      <c r="E89" t="s">
+        <v>127</v>
+      </c>
+      <c r="G89" t="s">
+        <v>125</v>
+      </c>
+      <c r="H89" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>8</v>
+      </c>
+      <c r="B90" s="1">
+        <v>46275.649305555547</v>
+      </c>
+      <c r="C90" s="3">
+        <v>5.5555555555555558E-3</v>
+      </c>
+      <c r="D90" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.654861111107</v>
+      </c>
+      <c r="E90" t="s">
+        <v>142</v>
+      </c>
+      <c r="G90" t="s">
+        <v>125</v>
+      </c>
+      <c r="H90" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>90</v>
+      </c>
+      <c r="B91" s="1">
+        <v>46275.654861111107</v>
+      </c>
+      <c r="C91" s="3">
+        <v>5.347222222222222E-2</v>
+      </c>
+      <c r="D91" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.708333333328</v>
+      </c>
+      <c r="E91" t="s">
+        <v>127</v>
+      </c>
+      <c r="G91" t="s">
+        <v>125</v>
+      </c>
+      <c r="H91" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>12</v>
+      </c>
+      <c r="B92" s="1">
+        <v>46275.708333333343</v>
+      </c>
+      <c r="C92" s="3">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D92" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46275.770833333343</v>
+      </c>
+      <c r="E92" t="s">
+        <v>25</v>
+      </c>
+      <c r="G92" t="s">
+        <v>125</v>
+      </c>
+      <c r="H92" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>8</v>
+      </c>
+      <c r="B93" s="1">
+        <v>46276.333333333343</v>
+      </c>
+      <c r="C93" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D93" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.336805555562</v>
+      </c>
+      <c r="E93" t="s">
+        <v>9</v>
+      </c>
+      <c r="G93" t="s">
+        <v>125</v>
+      </c>
+      <c r="H93" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>12</v>
+      </c>
+      <c r="B94" s="1">
+        <v>46276.336805555547</v>
+      </c>
+      <c r="C94" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D94" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.357638888883</v>
+      </c>
+      <c r="E94" t="s">
+        <v>147</v>
+      </c>
+      <c r="G94" t="s">
+        <v>125</v>
+      </c>
+      <c r="H94" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>90</v>
+      </c>
+      <c r="B95" s="1">
+        <v>46276.357638888891</v>
+      </c>
+      <c r="C95" s="3">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D95" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.399305555555</v>
+      </c>
+      <c r="E95" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>8</v>
+      </c>
+      <c r="B96" s="1">
+        <v>46276.399305555555</v>
+      </c>
+      <c r="C96" s="3">
+        <v>5.9027777777777776E-2</v>
+      </c>
+      <c r="D96" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.458333333336</v>
+      </c>
+      <c r="E96" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>8</v>
+      </c>
+      <c r="B97" s="1">
+        <v>46276.458333333336</v>
+      </c>
+      <c r="C97" s="3">
+        <v>1.3888888888888888E-2</v>
+      </c>
+      <c r="D97" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.472222222226</v>
+      </c>
+      <c r="E97" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>8</v>
+      </c>
+      <c r="B98" s="1">
+        <v>46276.472222222219</v>
+      </c>
+      <c r="C98" s="3">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="D98" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.479166666664</v>
+      </c>
+      <c r="E98" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>8</v>
+      </c>
+      <c r="B99" s="1">
+        <v>46276.479166666664</v>
+      </c>
+      <c r="C99" s="3">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="D99" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.489583333328</v>
+      </c>
+      <c r="E99" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>8</v>
+      </c>
+      <c r="B100" s="1">
+        <v>46276.489583333336</v>
+      </c>
+      <c r="C100" s="3">
+        <v>2.2222222222222223E-2</v>
+      </c>
+      <c r="D100" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.511805555558</v>
+      </c>
+      <c r="E100" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>12</v>
+      </c>
+      <c r="B101" s="1">
+        <v>46276.511805555558</v>
+      </c>
+      <c r="C101" s="3">
+        <v>0</v>
+      </c>
+      <c r="D101" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.511805555558</v>
+      </c>
+      <c r="E101" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>12</v>
+      </c>
+      <c r="B102" s="1">
+        <v>46276.666666666664</v>
+      </c>
+      <c r="C102" s="3">
+        <v>2.7777777777777776E-2</v>
+      </c>
+      <c r="D102" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.694444444445</v>
+      </c>
+      <c r="E102" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>153</v>
+      </c>
+      <c r="B103" s="1">
+        <v>46276.694444444445</v>
+      </c>
+      <c r="C103" s="3">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D103" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.715277777781</v>
+      </c>
+      <c r="E103" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>154</v>
+      </c>
+      <c r="B104" s="1">
+        <v>46276.715277777781</v>
+      </c>
+      <c r="C104" s="3">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D104" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.736111111117</v>
+      </c>
+      <c r="E104" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>157</v>
+      </c>
+      <c r="B105" s="1">
+        <v>46276.736111111109</v>
+      </c>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46276.736111111109</v>
       </c>
     </row>
   </sheetData>
@@ -2169,4 +3419,13 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
02_ventas correccion tipo de datos en ventas
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IRISCENE ENGINEERING CORPORATION SLU\Data Analytics Reporting Fractalia - CHILE\Miguel Paredes\Desarrollo\02. PYTHON\202_bot_jira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{150D6FB2-4E4C-497D-8BB6-B8549DA1098A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{113D18A8-856D-4D84-832F-E13DBF997A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="264">
   <si>
     <t>Ticket</t>
   </si>
@@ -741,22 +741,91 @@
     <t>514662</t>
   </si>
   <si>
+    <t>Sí (actualizado 21/09/2026 06:38)</t>
+  </si>
+  <si>
     <t>514663</t>
   </si>
   <si>
     <t>514664</t>
   </si>
   <si>
-    <t>Actualizar</t>
+    <t>Revision ETL de ventas dado que habia quiebres y fuentes rotas, se corrigio ello.</t>
+  </si>
+  <si>
+    <t>Sí (21/09/2026 06:38)</t>
+  </si>
+  <si>
+    <t>515322</t>
+  </si>
+  <si>
+    <t>515400</t>
   </si>
   <si>
     <t>Envio el archivo de comisiones</t>
   </si>
   <si>
-    <t>Revision ETL de ventas dado que habia quiebres y fuentes rotas, se corrigio ello.</t>
+    <t>515323</t>
   </si>
   <si>
     <t>Actualización CDM</t>
+  </si>
+  <si>
+    <t>515324</t>
+  </si>
+  <si>
+    <t>Actualización Dimensionado</t>
+  </si>
+  <si>
+    <t>515325</t>
+  </si>
+  <si>
+    <t>Actualización Accesos</t>
+  </si>
+  <si>
+    <t>515401</t>
+  </si>
+  <si>
+    <t>Actualizacion cartera al 15 de setiembre</t>
+  </si>
+  <si>
+    <t>515326</t>
+  </si>
+  <si>
+    <t>515402</t>
+  </si>
+  <si>
+    <t>Actualizacion dimensionado por cambio de asesor que pide descanso del miercoles al martes</t>
+  </si>
+  <si>
+    <t>515327</t>
+  </si>
+  <si>
+    <t>Actualizacion Comisiones por no considerar aquellas ventas que no ameritan comisionar</t>
+  </si>
+  <si>
+    <t>515403</t>
+  </si>
+  <si>
+    <t>515404</t>
+  </si>
+  <si>
+    <t>515406</t>
+  </si>
+  <si>
+    <t>DSS-9332</t>
+  </si>
+  <si>
+    <t>Se agregó el dominio @tigo al codigo como interno y dominio</t>
+  </si>
+  <si>
+    <t>Dimensionado</t>
+  </si>
+  <si>
+    <t>Actualización de cuartilizados (al pendiente por dos errores: faltan notas de calidad, faltas registros de logueo)</t>
+  </si>
+  <si>
+    <t>Autoevaluación teletrabajo, encuesta solicitada por el área de personas</t>
   </si>
 </sst>
 </file>
@@ -896,8 +965,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H152" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:H152" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla1" displayName="Tabla1" ref="A1:H166" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+  <autoFilter ref="A1:H166" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Ticket"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Fecha" dataDxfId="2"/>
@@ -1199,7 +1268,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
@@ -4722,26 +4791,23 @@
         <v>8</v>
       </c>
       <c r="B147" s="1">
-        <v>46282.270833333336</v>
+        <v>46282.270833333343</v>
       </c>
       <c r="C147" s="3">
         <v>3.472222222222222E-3</v>
       </c>
       <c r="D147" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46282.274305555555</v>
+        <v>46282.274305555562</v>
       </c>
       <c r="E147" t="s">
         <v>9</v>
       </c>
-      <c r="F147" t="s">
-        <v>237</v>
-      </c>
       <c r="G147" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="H147" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.25">
@@ -4765,7 +4831,7 @@
         <v>226</v>
       </c>
       <c r="H148" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.25">
@@ -4773,17 +4839,23 @@
         <v>8</v>
       </c>
       <c r="B149" s="1">
-        <v>46282.336805555555</v>
+        <v>46282.336805555547</v>
       </c>
       <c r="C149" s="3">
-        <v>0.12152777777777778</v>
+        <v>0.1215277777777778</v>
       </c>
       <c r="D149" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46282.458333333336</v>
+        <v>46282.458333333328</v>
       </c>
       <c r="E149" t="s">
+        <v>238</v>
+      </c>
+      <c r="G149" t="s">
         <v>239</v>
+      </c>
+      <c r="H149" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.25">
@@ -4791,18 +4863,24 @@
         <v>8</v>
       </c>
       <c r="B150" s="1">
-        <v>46279.458333333343</v>
+        <v>46282.458333333343</v>
       </c>
       <c r="C150" s="3">
         <v>1.388888888888889E-2</v>
       </c>
       <c r="D150" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46279.472222222234</v>
+        <v>46282.472222222234</v>
       </c>
       <c r="E150" t="s">
         <v>20</v>
       </c>
+      <c r="G150" t="s">
+        <v>239</v>
+      </c>
+      <c r="H150" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
@@ -4812,14 +4890,20 @@
         <v>46282.472222222219</v>
       </c>
       <c r="C151" s="3">
-        <v>1.0416666666666666E-2</v>
+        <v>1.041666666666667E-2</v>
       </c>
       <c r="D151" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
         <v>46282.482638888883</v>
       </c>
       <c r="E151" t="s">
-        <v>238</v>
+        <v>242</v>
+      </c>
+      <c r="G151" t="s">
+        <v>239</v>
+      </c>
+      <c r="H151" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
@@ -4830,14 +4914,320 @@
         <v>46282.482638888891</v>
       </c>
       <c r="C152" s="3">
-        <v>1.0416666666666666E-2</v>
+        <v>4.5138888888888888E-2</v>
       </c>
       <c r="D152" s="3">
         <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
-        <v>46282.493055555555</v>
+        <v>46282.527777777781</v>
       </c>
       <c r="E152" t="s">
-        <v>240</v>
+        <v>244</v>
+      </c>
+      <c r="G152" t="s">
+        <v>239</v>
+      </c>
+      <c r="H152" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>8</v>
+      </c>
+      <c r="B153" s="1">
+        <v>46282.527777777781</v>
+      </c>
+      <c r="C153" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D153" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.548611111117</v>
+      </c>
+      <c r="E153" t="s">
+        <v>246</v>
+      </c>
+      <c r="G153" t="s">
+        <v>239</v>
+      </c>
+      <c r="H153" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>8</v>
+      </c>
+      <c r="B154" s="1">
+        <v>46282.548611111109</v>
+      </c>
+      <c r="C154" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D154" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.552083333328</v>
+      </c>
+      <c r="E154" t="s">
+        <v>248</v>
+      </c>
+      <c r="G154" t="s">
+        <v>239</v>
+      </c>
+      <c r="H154" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>8</v>
+      </c>
+      <c r="B155" s="1">
+        <v>46282.542361111111</v>
+      </c>
+      <c r="C155" s="3">
+        <v>2.013888888888889E-2</v>
+      </c>
+      <c r="D155" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.5625</v>
+      </c>
+      <c r="E155" t="s">
+        <v>250</v>
+      </c>
+      <c r="G155" t="s">
+        <v>239</v>
+      </c>
+      <c r="H155" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>8</v>
+      </c>
+      <c r="B156" s="1">
+        <v>46282.5625</v>
+      </c>
+      <c r="C156" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D156" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.583333333336</v>
+      </c>
+      <c r="E156" t="s">
+        <v>244</v>
+      </c>
+      <c r="G156" t="s">
+        <v>239</v>
+      </c>
+      <c r="H156" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>8</v>
+      </c>
+      <c r="B157" s="1">
+        <v>46282.625</v>
+      </c>
+      <c r="C157" s="3">
+        <v>2.0833333333333329E-2</v>
+      </c>
+      <c r="D157" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.645833333336</v>
+      </c>
+      <c r="E157" t="s">
+        <v>253</v>
+      </c>
+      <c r="G157" t="s">
+        <v>239</v>
+      </c>
+      <c r="H157" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>8</v>
+      </c>
+      <c r="B158" s="1">
+        <v>46282.645833333343</v>
+      </c>
+      <c r="C158" s="3">
+        <v>1.7361111111111108E-2</v>
+      </c>
+      <c r="D158" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.663194444453</v>
+      </c>
+      <c r="E158" t="s">
+        <v>255</v>
+      </c>
+      <c r="G158" t="s">
+        <v>239</v>
+      </c>
+      <c r="H158" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>8</v>
+      </c>
+      <c r="B159" s="1">
+        <v>46282.663194444453</v>
+      </c>
+      <c r="C159" s="3">
+        <v>6.3194444444444442E-2</v>
+      </c>
+      <c r="D159" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46282.726388888899</v>
+      </c>
+      <c r="E159" t="s">
+        <v>244</v>
+      </c>
+      <c r="G159" t="s">
+        <v>239</v>
+      </c>
+      <c r="H159" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>8</v>
+      </c>
+      <c r="B160" s="1">
+        <v>46286.270833333343</v>
+      </c>
+      <c r="C160" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D160" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.274305555562</v>
+      </c>
+      <c r="E160" t="s">
+        <v>9</v>
+      </c>
+      <c r="G160" t="s">
+        <v>239</v>
+      </c>
+      <c r="H160" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>259</v>
+      </c>
+      <c r="B161" s="1">
+        <v>46286.274305555555</v>
+      </c>
+      <c r="C161" s="3">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D161" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.277777777774</v>
+      </c>
+      <c r="E161" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>8</v>
+      </c>
+      <c r="B162" s="1">
+        <v>46286.277777777781</v>
+      </c>
+      <c r="C162" s="3">
+        <v>5.9027777777777776E-2</v>
+      </c>
+      <c r="D162" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.336805555562</v>
+      </c>
+      <c r="E162" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>8</v>
+      </c>
+      <c r="B163" s="1">
+        <v>46286.336805555555</v>
+      </c>
+      <c r="C163" s="3">
+        <v>1.7361111111111112E-2</v>
+      </c>
+      <c r="D163" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.354166666664</v>
+      </c>
+      <c r="E163" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>12</v>
+      </c>
+      <c r="B164" s="1">
+        <v>46286.354166666664</v>
+      </c>
+      <c r="C164" s="3">
+        <v>0</v>
+      </c>
+      <c r="D164" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.354166666664</v>
+      </c>
+      <c r="E164" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>12</v>
+      </c>
+      <c r="B165" s="1">
+        <v>46286.375</v>
+      </c>
+      <c r="C165" s="3">
+        <v>1.7361111111111112E-2</v>
+      </c>
+      <c r="D165" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.392361111109</v>
+      </c>
+      <c r="E165" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>12</v>
+      </c>
+      <c r="B166" s="1">
+        <v>46286.375</v>
+      </c>
+      <c r="C166" s="3">
+        <v>1.7361111111111112E-2</v>
+      </c>
+      <c r="D166" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v>46286.392361111109</v>
+      </c>
+      <c r="E166" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
11_correos se agregó el modelo bronce - gold -silver
</commit_message>
<xml_diff>
--- a/202_bot_jira/worklog.xlsx
+++ b/202_bot_jira/worklog.xlsx
@@ -209,8 +209,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H182" headerRowCount="1" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
-  <autoFilter ref="A1:H182"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="A1:H193" headerRowCount="1" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+  <autoFilter ref="A1:H193"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Ticket"/>
     <tableColumn id="2" name="Fecha" dataDxfId="2"/>
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H182"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="18.140625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -6540,6 +6540,369 @@
       <c r="H182" t="inlineStr">
         <is>
           <t>516312</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>DSS-9756</t>
+        </is>
+      </c>
+      <c r="B183" s="1" t="n">
+        <v>46288.27430555555</v>
+      </c>
+      <c r="C183" s="3" t="n">
+        <v>0.06736111111111111</v>
+      </c>
+      <c r="D183" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Desarrollo bronce</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>516595</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>DSS-9337</t>
+        </is>
+      </c>
+      <c r="B184" s="1" t="n">
+        <v>46288.34166666667</v>
+      </c>
+      <c r="C184" s="3" t="n">
+        <v>0.01041666666666667</v>
+      </c>
+      <c r="D184" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Llamada de Diego para revisar el proceso de descarga de base de agentes del portal comercial</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>516596</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B185" s="1" t="n">
+        <v>46288.35208333333</v>
+      </c>
+      <c r="C185" s="3" t="n">
+        <v>0.02291666666666667</v>
+      </c>
+      <c r="D185" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Desarrollo bot descarga agentes del portal comercial</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>516699</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>DSS-9337</t>
+        </is>
+      </c>
+      <c r="B186" s="1" t="n">
+        <v>46288.375</v>
+      </c>
+      <c r="C186" s="3" t="n">
+        <v>0.02083333333333333</v>
+      </c>
+      <c r="D186" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>516597</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B187" s="1" t="n">
+        <v>46288.39583333334</v>
+      </c>
+      <c r="C187" s="3" t="n">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="D187" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Desarrollo bot descarga agentes del portal comercial</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>516700</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B188" s="1" t="n">
+        <v>46288.47916666666</v>
+      </c>
+      <c r="C188" s="3" t="n">
+        <v>0.01041666666666667</v>
+      </c>
+      <c r="D188" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Corrida ETL tráfico, calidad, usuarios chile</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>516701</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B189" s="1" t="n">
+        <v>46288.48958333334</v>
+      </c>
+      <c r="C189" s="3" t="n">
+        <v>0.09375</v>
+      </c>
+      <c r="D189" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Desarrollo bot descarga agentes del portal comercial</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>516598</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>DSS-9756</t>
+        </is>
+      </c>
+      <c r="B190" s="1" t="n">
+        <v>46288.625</v>
+      </c>
+      <c r="C190" s="3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="D190" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Desarrollo ETL silver y gold</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>516702</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>DSS-9336</t>
+        </is>
+      </c>
+      <c r="B191" s="1" t="n">
+        <v>46289.27083333334</v>
+      </c>
+      <c r="C191" s="3" t="n">
+        <v>0.003472222222222222</v>
+      </c>
+      <c r="D191" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Descarga insumos SF</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>516599</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>DSS-9756</t>
+        </is>
+      </c>
+      <c r="B192" s="1" t="n">
+        <v>46288.27430555555</v>
+      </c>
+      <c r="C192" s="3" t="n">
+        <v>0.1006944444444444</v>
+      </c>
+      <c r="D192" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Desarrollo ETL hechos y dimensiones</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>516703</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>DSS-9337</t>
+        </is>
+      </c>
+      <c r="B193" s="1" t="n">
+        <v>46288.375</v>
+      </c>
+      <c r="C193" s="3" t="n">
+        <v>0.01041666666666667</v>
+      </c>
+      <c r="D193" s="3">
+        <f>Tabla1[[#This Row],[Fecha]]+Tabla1[[#This Row],[Horas]]</f>
+        <v/>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Sí (24/09/2026 10:04)</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>516800</t>
         </is>
       </c>
     </row>

</xml_diff>